<commit_message>
Fix two instructions in the sprint workbook README
The daily-use line told the team to type into blue cells while the legend two
rows below said yellow. Inputs are yellow-filled with blue text, so the legend
was right and the instruction was wrong.

The v4 source citation pointed at 10_KPIs_By_GE. The sheet renumbering pass
that shifted this workbook's own tabs also caught the citation string; v4 ships
09_KPIs_By_GE.
</commit_message>
<xml_diff>
--- a/workbooks/bridgeapp_qualifying_sprint_20260824_v1.xlsx
+++ b/workbooks/bridgeapp_qualifying_sprint_20260824_v1.xlsx
@@ -764,7 +764,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>The named owner fills yesterday's row in 05_Daily_Log. Blue cells are the only cells anyone types into.</t>
+          <t>The named owner fills yesterday's row in 05_Daily_Log. Yellow cells are the only cells anyone types into.</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
     <row r="31">
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Source for all pre-filled targets and budget lines: BridgeApp Phase 2 Operating Workbook v4 (May 2026), sheets 02_Budget_Master, 03_Calendar_Phase2, 04_GE1_Tracker, 05_GE2_Tracker, 10_KPIs_By_GE.</t>
+          <t>Source for all pre-filled targets and budget lines: BridgeApp Phase 2 Operating Workbook v4 (May 2026), sheets 02_Budget_Master, 03_Calendar_Phase2, 04_GE1_Tracker, 05_GE2_Tracker, 09_KPIs_By_GE.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Move sales counting from the Campaign Lead to Gradesmatch tech
The daily Peach reconciliation is not resourced on the growth side, so it
becomes a tech function. That changes more than an owner column: manual
reconciliation was the stated fallback for the GA4 purchase event not landing,
so the fallback no longer exists.

Counting a sale now needs either the purchase event or an automated feed of
cleared transactions. The feed is added as a fourth dev dependency and promoted
from a scale limit to a blocker in the report, and the claim that the sprint
still runs on manual reconciliation is removed from all three documents.

Also created a shared daily-log capture sheet in Drive, and confirmed by test
that formulas do not survive the CSV upload path, so the pace line ships as
pre-computed values rather than a promise the sheet cannot keep.
</commit_message>
<xml_diff>
--- a/workbooks/bridgeapp_qualifying_sprint_20260824_v1.xlsx
+++ b/workbooks/bridgeapp_qualifying_sprint_20260824_v1.xlsx
@@ -1029,7 +1029,7 @@
     <row r="33">
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Sales in this sprint are counted from the Peach transaction export reconciled against the ledger. GA4 cannot attribute a sale until the purchase event is installed. See 03_Sprint_Drivers row 24.</t>
+          <t>Counting sales is a Gradesmatch tech function, not a manual task. It needs either the GA4 purchase event or an automated feed of cleared Peach transactions. Until one of them lands, this workbook has no way to record a sale. See 03_Sprint_Drivers.</t>
         </is>
       </c>
     </row>
@@ -2544,7 +2544,7 @@
     <row r="26">
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Peach reconciled to ledger by 09:00</t>
+          <t>Peach feed landing daily</t>
         </is>
       </c>
       <c r="C26" s="37" t="inlineStr">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>Campaign Lead</t>
+          <t>Gradesmatch tech</t>
         </is>
       </c>
       <c r="F26" s="72" t="inlineStr">
@@ -3476,12 +3476,12 @@
     <row r="17">
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Peach reconciliation to ledger</t>
+          <t>Sales counting, Peach to ledger</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Campaign Lead</t>
+          <t>Gradesmatch tech</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Daily by 09:00</t>
+          <t>Automated, daily</t>
         </is>
       </c>
     </row>
@@ -4848,7 +4848,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E56"/>
+  <dimension ref="B2:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -5399,7 +5399,7 @@
       </c>
       <c r="C46" s="21" t="inlineStr">
         <is>
-          <t>Peach transaction export, reconciled against the sales ledger daily by 09:00 by the Campaign Lead.</t>
+          <t>An automated feed of cleared Peach transactions, delivered by Gradesmatch tech. This is a tech function. Nobody on the growth team has capacity to reconcile by hand every day.</t>
         </is>
       </c>
     </row>
@@ -5492,7 +5492,7 @@
       </c>
       <c r="E54" s="33" t="inlineStr">
         <is>
-          <t>Sprint runs on manual Peach reconciliation. Cost per sale is still measurable. Channel attribution is weaker.</t>
+          <t>Without this OR the transaction feed below, no sale can be recorded at all and the sprint measures nothing. With the feed but not this, sales are counted but cannot be split by channel.</t>
         </is>
       </c>
     </row>
@@ -5527,6 +5527,23 @@
       <c r="E56" s="33" t="inlineStr">
         <is>
           <t>Readiness tracker submissions are not captured, so click to signup stays unmeasured and only click to sale can be read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="26" customHeight="1">
+      <c r="B57" s="32" t="inlineStr">
+        <is>
+          <t>Automated feed of cleared Peach transactions</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>Day 1, 24 Aug</t>
+        </is>
+      </c>
+      <c r="E57" s="33" t="inlineStr">
+        <is>
+          <t>The manual reconciliation this replaces is no longer resourced. Without this or the purchase event there is no way to count a sale.</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5768,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Baseline: closing Peach ledger count recorded in 05_Daily_Log</t>
+          <t>Baseline: closing sales count recorded in 05_Daily_Log</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -5769,9 +5786,9 @@
           <t>PLANNED</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Sprint</t>
+      <c r="I10" s="22" t="inlineStr">
+        <is>
+          <t>Blocked: dev</t>
         </is>
       </c>
     </row>
@@ -6180,7 +6197,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Mid week reconciliation check against Peach</t>
+          <t>Mid week check that the Peach feed is landing</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -7050,7 +7067,7 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Final Peach reconciliation for the sprint</t>
+          <t>Final sales count confirmed against the Peach feed</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
@@ -7068,9 +7085,9 @@
           <t>PLANNED</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>Sprint</t>
+      <c r="I46" s="22" t="inlineStr">
+        <is>
+          <t>Blocked: dev</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Resolve the two UTM registers down to one, and document the surface split
Tab 09_UTM_Register duplicated the standalone UTM link builder Sheet, formulas
and all, so links could be tagged in one place and counted from the other. The
Sheet wins: the team already uses it, it is in Drive, and a workbook file gets
emailed and forked. The tab is now a checklist of the codes this sprint needs
with a tick column, and the KPI counts ticks rather than built URLs.

Also corrected stale codes on that tab. It still carried school-kingsmead and
sahisa-durban from the Phase 2 calendar; the real schools are Pretoria
Technical, Pretoria-Wes and Pretoria Girls.

README now states the architecture plainly: Sheets for capture because the team
edits them, the workbook for the model because one person owns it and it needs
formulas. Forcing both into one file is what breaks.

1 530 formula cells, zero errors.
</commit_message>
<xml_diff>
--- a/workbooks/bridgeapp_qualifying_sprint_20260824_v1.xlsx
+++ b/workbooks/bridgeapp_qualifying_sprint_20260824_v1.xlsx
@@ -122,7 +122,7 @@
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="FF0B1220"/>
+      <color rgb="FF4A90D9"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -181,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -329,7 +329,10 @@
     <xf numFmtId="2" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="7" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1044,40 +1047,39 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:K23"/>
+  <dimension ref="B2:J32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="74" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="2" ht="27" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>UTM REGISTER</t>
+          <t>UTM CODES</t>
         </is>
       </c>
     </row>
     <row r="3" ht="13" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Every link used in the sprint. A link that is not on this sheet cannot be attributed, so the sale it produces counts for nobody.</t>
+          <t>There is one live register and it is not this tab. Links are built and stored in the BridgeApp UTM link builder in Google Drive, so the whole team works off one list.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Type into the yellow cells. Column H builds itself</t>
+          <t>Where links live</t>
         </is>
       </c>
       <c r="C5" s="4" t="n"/>
@@ -1087,689 +1089,680 @@
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="n"/>
       <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
-    </row>
-    <row r="6" ht="26" customHeight="1">
-      <c r="B6" s="11" t="inlineStr">
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Live register</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>BridgeApp UTM link builder, Google Sheets. Every link is created there and nowhere else.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="C7" s="63" t="inlineStr">
+        <is>
+          <t>https://docs.google.com/spreadsheets/d/1D7rVlQW8ym0bb20i3-7qmEHBS5fxVVRegwjdhaK9JF8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Why not here</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>A workbook file gets emailed and forked. A Sheet does not. Two registers means links tagged in one and counted from the other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>This tab</t>
+        </is>
+      </c>
+      <c r="C9" s="21" t="inlineStr">
+        <is>
+          <t>The checklist of codes this sprint needs. Tick each one off as it is created in the register.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Codes this sprint needs. Tick column H when it exists in the live register.</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Campaign</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F12" s="11" t="inlineStr">
         <is>
           <t>Content</t>
         </is>
       </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>Landing URL</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>Tagged URL, copy this one</t>
-        </is>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>GE</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>Created? Y/N</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="K6" s="11" t="inlineStr">
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>Live from</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>Meta paid, parent audience</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>meta</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>paid-social</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>qualifying-sprint</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>meta-set-a</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H7" s="63">
-        <f>IF(OR(G7="",C7="",D7=""),"",G7&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C7))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D7))," ","-"),"/","-"),"--","-")&amp;IF(E7="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E7))," ","-"),"/","-"),"--","-"))&amp;IF(F7="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F7))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I7" s="41" t="inlineStr">
-        <is>
-          <t>GE1</t>
-        </is>
-      </c>
-      <c r="J7" s="12" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="K7" s="64" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Meta paid, retargeting July leads</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>meta</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>paid-social</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>qualifying-sprint</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>meta-retarget</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H8" s="63">
-        <f>IF(OR(G8="",C8="",D8=""),"",G8&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C8))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D8))," ","-"),"/","-"),"--","-")&amp;IF(E8="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E8))," ","-"),"/","-"),"--","-"))&amp;IF(F8="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F8))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I8" s="41" t="inlineStr">
-        <is>
-          <t>GE1</t>
-        </is>
-      </c>
-      <c r="J8" s="12" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="K8" s="64" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Google paid search, brand</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>google</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>paid-search</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>qualifying-sprint</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>brand</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H9" s="63">
-        <f>IF(OR(G9="",C9="",D9=""),"",G9&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C9))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D9))," ","-"),"/","-"),"--","-")&amp;IF(E9="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E9))," ","-"),"/","-"),"--","-"))&amp;IF(F9="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F9))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I9" s="41" t="inlineStr">
-        <is>
-          <t>GE1</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="K9" s="64" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>LinkedIn paid, school leaders</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>paid-social</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>qualifying-sprint</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>school-leaders</t>
-        </is>
-      </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H10" s="63">
-        <f>IF(OR(G10="",C10="",D10=""),"",G10&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C10))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D10))," ","-"),"/","-"),"--","-")&amp;IF(E10="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E10))," ","-"),"/","-"),"--","-"))&amp;IF(F10="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F10))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I10" s="41" t="inlineStr">
-        <is>
-          <t>GE1</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="K10" s="64" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>Boosted organic, best of last week</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>facebook</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>boosted</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>qualifying-sprint</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>weekly-boost</t>
-        </is>
-      </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H11" s="63">
-        <f>IF(OR(G11="",C11="",D11=""),"",G11&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C11))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D11))," ","-"),"/","-"),"--","-")&amp;IF(E11="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E11))," ","-"),"/","-"),"--","-"))&amp;IF(F11="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F11))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I11" s="41" t="inlineStr">
-        <is>
-          <t>GE1</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="K11" s="64" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Influencer Wave 3, GP creator</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>influencer</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>referral</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>qualifying-sprint</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>wave-3-gp</t>
-        </is>
-      </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H12" s="63">
-        <f>IF(OR(G12="",C12="",D12=""),"",G12&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C12))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D12))," ","-"),"/","-"),"--","-")&amp;IF(E12="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E12))," ","-"),"/","-"),"--","-"))&amp;IF(F12="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F12))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I12" s="41" t="inlineStr">
-        <is>
-          <t>GE1</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="inlineStr">
-        <is>
-          <t>TBC</t>
-        </is>
-      </c>
-      <c r="K12" s="64" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Instagram bio link</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>instagram</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>organic-social</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
+          <t>Meta paid, parent audience</t>
+        </is>
+      </c>
+      <c r="C13" s="64" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="D13" s="64" t="inlineStr">
+        <is>
+          <t>paid-social</t>
+        </is>
+      </c>
+      <c r="E13" s="64" t="inlineStr">
         <is>
           <t>qualifying-sprint</t>
         </is>
       </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>bio-link</t>
-        </is>
-      </c>
-      <c r="G13" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H13" s="63">
-        <f>IF(OR(G13="",C13="",D13=""),"",G13&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C13))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D13))," ","-"),"/","-"),"--","-")&amp;IF(E13="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E13))," ","-"),"/","-"),"--","-"))&amp;IF(F13="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F13))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I13" s="41" t="inlineStr">
+      <c r="F13" s="64" t="inlineStr">
+        <is>
+          <t>meta-set-a</t>
+        </is>
+      </c>
+      <c r="G13" s="41" t="inlineStr">
         <is>
           <t>GE1</t>
         </is>
       </c>
-      <c r="J13" s="12" t="inlineStr">
+      <c r="H13" s="40" t="n"/>
+      <c r="I13" s="12" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="K13" s="64" t="n"/>
+      <c r="J13" s="65" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>WhatsApp concierge broadcast</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>whatsapp</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>message</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
+          <t>Meta paid, retargeting July leads</t>
+        </is>
+      </c>
+      <c r="C14" s="64" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="D14" s="64" t="inlineStr">
+        <is>
+          <t>paid-social</t>
+        </is>
+      </c>
+      <c r="E14" s="64" t="inlineStr">
         <is>
           <t>qualifying-sprint</t>
         </is>
       </c>
-      <c r="F14" s="12" t="inlineStr">
-        <is>
-          <t>broadcast</t>
-        </is>
-      </c>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H14" s="63">
-        <f>IF(OR(G14="",C14="",D14=""),"",G14&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C14))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D14))," ","-"),"/","-"),"--","-")&amp;IF(E14="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E14))," ","-"),"/","-"),"--","-"))&amp;IF(F14="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F14))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I14" s="41" t="inlineStr">
+      <c r="F14" s="64" t="inlineStr">
+        <is>
+          <t>meta-retarget</t>
+        </is>
+      </c>
+      <c r="G14" s="41" t="inlineStr">
         <is>
           <t>GE1</t>
         </is>
       </c>
-      <c r="J14" s="12" t="inlineStr">
+      <c r="H14" s="40" t="n"/>
+      <c r="I14" s="12" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="K14" s="64" t="n"/>
+      <c r="J14" s="65" t="n"/>
     </row>
     <row r="15">
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Nurture emailer</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
+          <t>Meta paid, 20 second recut</t>
+        </is>
+      </c>
+      <c r="C15" s="64" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="D15" s="64" t="inlineStr">
+        <is>
+          <t>paid-social</t>
+        </is>
+      </c>
+      <c r="E15" s="64" t="inlineStr">
         <is>
           <t>qualifying-sprint</t>
         </is>
       </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>nurture-1</t>
-        </is>
-      </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H15" s="63">
-        <f>IF(OR(G15="",C15="",D15=""),"",G15&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C15))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D15))," ","-"),"/","-"),"--","-")&amp;IF(E15="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E15))," ","-"),"/","-"),"--","-"))&amp;IF(F15="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F15))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I15" s="41" t="inlineStr">
+      <c r="F15" s="64" t="inlineStr">
+        <is>
+          <t>recut-20s</t>
+        </is>
+      </c>
+      <c r="G15" s="41" t="inlineStr">
         <is>
           <t>GE1</t>
         </is>
       </c>
-      <c r="J15" s="12" t="inlineStr">
+      <c r="H15" s="40" t="n"/>
+      <c r="I15" s="12" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="K15" s="64" t="n"/>
+      <c r="J15" s="65" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>School visit QR, generic</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>school-visits</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>qr</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
+          <t>Meta paid, static statement</t>
+        </is>
+      </c>
+      <c r="C16" s="64" t="inlineStr">
+        <is>
+          <t>meta</t>
+        </is>
+      </c>
+      <c r="D16" s="64" t="inlineStr">
+        <is>
+          <t>paid-social</t>
+        </is>
+      </c>
+      <c r="E16" s="64" t="inlineStr">
         <is>
           <t>qualifying-sprint</t>
         </is>
       </c>
-      <c r="F16" s="12" t="inlineStr"/>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H16" s="63">
-        <f>IF(OR(G16="",C16="",D16=""),"",G16&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C16))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D16))," ","-"),"/","-"),"--","-")&amp;IF(E16="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E16))," ","-"),"/","-"),"--","-"))&amp;IF(F16="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F16))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I16" s="42" t="inlineStr">
-        <is>
-          <t>GE2</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="inlineStr">
+      <c r="F16" s="64" t="inlineStr">
+        <is>
+          <t>static-statement</t>
+        </is>
+      </c>
+      <c r="G16" s="41" t="inlineStr">
+        <is>
+          <t>GE1</t>
+        </is>
+      </c>
+      <c r="H16" s="40" t="n"/>
+      <c r="I16" s="12" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="K16" s="64" t="n"/>
+      <c r="J16" s="65" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>School visit QR, per school</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>school-visits</t>
-        </is>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>qr</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="inlineStr">
+          <t>Boosted organic, best of last week</t>
+        </is>
+      </c>
+      <c r="C17" s="64" t="inlineStr">
+        <is>
+          <t>facebook</t>
+        </is>
+      </c>
+      <c r="D17" s="64" t="inlineStr">
+        <is>
+          <t>boosted</t>
+        </is>
+      </c>
+      <c r="E17" s="64" t="inlineStr">
         <is>
           <t>qualifying-sprint</t>
         </is>
       </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>school-kingsmead</t>
-        </is>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H17" s="63">
-        <f>IF(OR(G17="",C17="",D17=""),"",G17&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C17))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D17))," ","-"),"/","-"),"--","-")&amp;IF(E17="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E17))," ","-"),"/","-"),"--","-"))&amp;IF(F17="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F17))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I17" s="42" t="inlineStr">
-        <is>
-          <t>GE2</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="inlineStr">
+      <c r="F17" s="64" t="inlineStr">
+        <is>
+          <t>weekly-boost</t>
+        </is>
+      </c>
+      <c r="G17" s="41" t="inlineStr">
+        <is>
+          <t>GE1</t>
+        </is>
+      </c>
+      <c r="H17" s="40" t="n"/>
+      <c r="I17" s="12" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="K17" s="64" t="n"/>
+      <c r="J17" s="65" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Exhibition and conference QR</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="inlineStr">
-        <is>
-          <t>school-events</t>
-        </is>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>qr</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="inlineStr">
+          <t>Instagram bio link</t>
+        </is>
+      </c>
+      <c r="C18" s="64" t="inlineStr">
+        <is>
+          <t>instagram</t>
+        </is>
+      </c>
+      <c r="D18" s="64" t="inlineStr">
+        <is>
+          <t>organic-social</t>
+        </is>
+      </c>
+      <c r="E18" s="64" t="inlineStr">
         <is>
           <t>qualifying-sprint</t>
         </is>
       </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>sahisa-durban</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H18" s="63">
-        <f>IF(OR(G18="",C18="",D18=""),"",G18&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C18))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D18))," ","-"),"/","-"),"--","-")&amp;IF(E18="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E18))," ","-"),"/","-"),"--","-"))&amp;IF(F18="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F18))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I18" s="42" t="inlineStr">
-        <is>
-          <t>GE2</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="inlineStr">
+      <c r="F18" s="64" t="inlineStr">
+        <is>
+          <t>bio-link</t>
+        </is>
+      </c>
+      <c r="G18" s="41" t="inlineStr">
+        <is>
+          <t>GE1</t>
+        </is>
+      </c>
+      <c r="H18" s="40" t="n"/>
+      <c r="I18" s="12" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="K18" s="64" t="n"/>
+      <c r="J18" s="65" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Parent info session handout</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
+          <t>Nurture emailer</t>
+        </is>
+      </c>
+      <c r="C19" s="64" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="D19" s="64" t="inlineStr">
+        <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="E19" s="64" t="inlineStr">
+        <is>
+          <t>qualifying-sprint</t>
+        </is>
+      </c>
+      <c r="F19" s="64" t="inlineStr">
+        <is>
+          <t>nurture-1</t>
+        </is>
+      </c>
+      <c r="G19" s="41" t="inlineStr">
+        <is>
+          <t>GE1</t>
+        </is>
+      </c>
+      <c r="H19" s="40" t="n"/>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="J19" s="65" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>School QR, Pretoria Technical</t>
+        </is>
+      </c>
+      <c r="C20" s="64" t="inlineStr">
         <is>
           <t>school-visits</t>
         </is>
       </c>
-      <c r="D19" s="12" t="inlineStr">
+      <c r="D20" s="64" t="inlineStr">
+        <is>
+          <t>qr</t>
+        </is>
+      </c>
+      <c r="E20" s="64" t="inlineStr">
+        <is>
+          <t>qualifying-sprint</t>
+        </is>
+      </c>
+      <c r="F20" s="64" t="inlineStr">
+        <is>
+          <t>school-pretoria-technical</t>
+        </is>
+      </c>
+      <c r="G20" s="42" t="inlineStr">
+        <is>
+          <t>GE2</t>
+        </is>
+      </c>
+      <c r="H20" s="40" t="n"/>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="J20" s="65" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>School QR, Pretoria-Wes</t>
+        </is>
+      </c>
+      <c r="C21" s="64" t="inlineStr">
+        <is>
+          <t>school-visits</t>
+        </is>
+      </c>
+      <c r="D21" s="64" t="inlineStr">
+        <is>
+          <t>qr</t>
+        </is>
+      </c>
+      <c r="E21" s="64" t="inlineStr">
+        <is>
+          <t>qualifying-sprint</t>
+        </is>
+      </c>
+      <c r="F21" s="64" t="inlineStr">
+        <is>
+          <t>school-pretoria-wes</t>
+        </is>
+      </c>
+      <c r="G21" s="42" t="inlineStr">
+        <is>
+          <t>GE2</t>
+        </is>
+      </c>
+      <c r="H21" s="40" t="n"/>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="J21" s="65" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>School QR, Pretoria Girls</t>
+        </is>
+      </c>
+      <c r="C22" s="64" t="inlineStr">
+        <is>
+          <t>school-visits</t>
+        </is>
+      </c>
+      <c r="D22" s="64" t="inlineStr">
+        <is>
+          <t>qr</t>
+        </is>
+      </c>
+      <c r="E22" s="64" t="inlineStr">
+        <is>
+          <t>qualifying-sprint</t>
+        </is>
+      </c>
+      <c r="F22" s="64" t="inlineStr">
+        <is>
+          <t>school-pretoria-girls</t>
+        </is>
+      </c>
+      <c r="G22" s="42" t="inlineStr">
+        <is>
+          <t>GE2</t>
+        </is>
+      </c>
+      <c r="H22" s="40" t="n"/>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="J22" s="65" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>School QR, generic fallback</t>
+        </is>
+      </c>
+      <c r="C23" s="64" t="inlineStr">
+        <is>
+          <t>school-visits</t>
+        </is>
+      </c>
+      <c r="D23" s="64" t="inlineStr">
+        <is>
+          <t>qr</t>
+        </is>
+      </c>
+      <c r="E23" s="64" t="inlineStr">
+        <is>
+          <t>qualifying-sprint</t>
+        </is>
+      </c>
+      <c r="F23" s="64" t="inlineStr"/>
+      <c r="G23" s="42" t="inlineStr">
+        <is>
+          <t>GE2</t>
+        </is>
+      </c>
+      <c r="H23" s="40" t="n"/>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="J23" s="65" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Learner leave behind, printed</t>
+        </is>
+      </c>
+      <c r="C24" s="64" t="inlineStr">
+        <is>
+          <t>school-visits</t>
+        </is>
+      </c>
+      <c r="D24" s="64" t="inlineStr">
         <is>
           <t>print</t>
         </is>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="E24" s="64" t="inlineStr">
         <is>
           <t>qualifying-sprint</t>
         </is>
       </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>info-session</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
-        <is>
-          <t>https://bridgeapp.co.za/uniapply-parents</t>
-        </is>
-      </c>
-      <c r="H19" s="63">
-        <f>IF(OR(G19="",C19="",D19=""),"",G19&amp;"?utm_source="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(C19))," ","-"),"/","-"),"--","-")&amp;"&amp;utm_medium="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(D19))," ","-"),"/","-"),"--","-")&amp;IF(E19="","","&amp;utm_campaign="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(E19))," ","-"),"/","-"),"--","-"))&amp;IF(F19="","","&amp;utm_content="&amp;SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LOWER(TRIM(F19))," ","-"),"/","-"),"--","-")))</f>
-        <v/>
-      </c>
-      <c r="I19" s="42" t="inlineStr">
+      <c r="F24" s="64" t="inlineStr">
+        <is>
+          <t>leave-behind</t>
+        </is>
+      </c>
+      <c r="G24" s="42" t="inlineStr">
         <is>
           <t>GE2</t>
         </is>
       </c>
-      <c r="J19" s="12" t="inlineStr">
+      <c r="H24" s="40" t="n"/>
+      <c r="I24" s="12" t="inlineStr">
         <is>
           <t>TBC</t>
         </is>
       </c>
-      <c r="K19" s="64" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Landing URL is pre-filled with the parent page path. If the page is not deployed by day 1, change column G to the live destination on every row before any spend starts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Source and medium are compulsory. Campaign and content are optional and the formula leaves them out when blank.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Everything is forced to lower case with spaces turned into hyphens, because GA4 treats Meta and meta as two different sources.</t>
+      <c r="J24" s="65" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Parent take home slip</t>
+        </is>
+      </c>
+      <c r="C25" s="64" t="inlineStr">
+        <is>
+          <t>school-visits</t>
+        </is>
+      </c>
+      <c r="D25" s="64" t="inlineStr">
+        <is>
+          <t>print</t>
+        </is>
+      </c>
+      <c r="E25" s="64" t="inlineStr">
+        <is>
+          <t>qualifying-sprint</t>
+        </is>
+      </c>
+      <c r="F25" s="64" t="inlineStr">
+        <is>
+          <t>parent-slip</t>
+        </is>
+      </c>
+      <c r="G25" s="42" t="inlineStr">
+        <is>
+          <t>GE2</t>
+        </is>
+      </c>
+      <c r="H25" s="40" t="n"/>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>TBC</t>
+        </is>
+      </c>
+      <c r="J25" s="65" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Rules</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Source and medium are compulsory. Campaign and content are optional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Everything is lower case with spaces as hyphens, because GA4 treats Meta and meta as two different sources.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>The landing URL is the parent page. If it is not deployed, repoint every link in the register before any spend starts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>A school visited without its own code produces sales nobody can trace back to the room it started in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>A link that is not in the live register cannot be attributed, so the sale it produces counts for nobody.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="B29:J29"/>
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="B28:J28"/>
+    <mergeCell ref="C6:J6"/>
+    <mergeCell ref="B32:J32"/>
+    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B30:J30"/>
+    <mergeCell ref="C8:J8"/>
+    <mergeCell ref="C9:J9"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1895,11 +1888,11 @@
         <f>'06_GE1_Paid_Media'!$C$11</f>
         <v/>
       </c>
-      <c r="G7" s="65">
+      <c r="G7" s="66">
         <f>'03_Sprint_Drivers'!$C$26</f>
         <v/>
       </c>
-      <c r="H7" s="66">
+      <c r="H7" s="67">
         <f>'03_Sprint_Drivers'!$C$26*2</f>
         <v/>
       </c>
@@ -1938,11 +1931,11 @@
         <f>'06_GE1_Paid_Media'!$C$10</f>
         <v/>
       </c>
-      <c r="G8" s="67">
+      <c r="G8" s="68">
         <f>'03_Sprint_Drivers'!$C$17</f>
         <v/>
       </c>
-      <c r="H8" s="68">
+      <c r="H8" s="69">
         <f>ROUND('03_Sprint_Drivers'!$C$17*0.5,0)</f>
         <v/>
       </c>
@@ -1981,10 +1974,10 @@
         <f>'06_GE1_Paid_Media'!$C$12</f>
         <v/>
       </c>
-      <c r="G9" s="65" t="n">
+      <c r="G9" s="66" t="n">
         <v>85</v>
       </c>
-      <c r="H9" s="66" t="n">
+      <c r="H9" s="67" t="n">
         <v>120</v>
       </c>
       <c r="I9" s="47" t="inlineStr">
@@ -2025,7 +2018,7 @@
       <c r="G10" s="31" t="n">
         <v>0.04</v>
       </c>
-      <c r="H10" s="69" t="n">
+      <c r="H10" s="70" t="n">
         <v>0.025</v>
       </c>
       <c r="I10" s="47" t="inlineStr">
@@ -2063,10 +2056,10 @@
         <f>'06_GE1_Paid_Media'!$C$15</f>
         <v/>
       </c>
-      <c r="G11" s="65" t="n">
+      <c r="G11" s="66" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="66" t="n">
+      <c r="H11" s="67" t="n">
         <v>0</v>
       </c>
       <c r="I11" s="47" t="inlineStr">
@@ -2165,11 +2158,11 @@
         <f>'07_GE2_School_Outreach'!$C$11</f>
         <v/>
       </c>
-      <c r="G15" s="67">
+      <c r="G15" s="68">
         <f>'03_Sprint_Drivers'!$C$18</f>
         <v/>
       </c>
-      <c r="H15" s="68">
+      <c r="H15" s="69">
         <f>ROUND('03_Sprint_Drivers'!$C$18*0.5,0)</f>
         <v/>
       </c>
@@ -2208,11 +2201,11 @@
         <f>'07_GE2_School_Outreach'!$C$24</f>
         <v/>
       </c>
-      <c r="G16" s="65">
+      <c r="G16" s="66">
         <f>'03_Sprint_Drivers'!$C$26</f>
         <v/>
       </c>
-      <c r="H16" s="66">
+      <c r="H16" s="67">
         <f>'03_Sprint_Drivers'!$C$26*2</f>
         <v/>
       </c>
@@ -2251,10 +2244,10 @@
         <f>'07_GE2_School_Outreach'!$C$7</f>
         <v/>
       </c>
-      <c r="G17" s="67" t="n">
+      <c r="G17" s="68" t="n">
         <v>12</v>
       </c>
-      <c r="H17" s="68" t="n">
+      <c r="H17" s="69" t="n">
         <v>8</v>
       </c>
       <c r="I17" s="47" t="inlineStr">
@@ -2292,10 +2285,10 @@
         <f>'07_GE2_School_Outreach'!$C$9</f>
         <v/>
       </c>
-      <c r="G18" s="67" t="n">
+      <c r="G18" s="68" t="n">
         <v>50</v>
       </c>
-      <c r="H18" s="68" t="n">
+      <c r="H18" s="69" t="n">
         <v>30</v>
       </c>
       <c r="I18" s="47" t="inlineStr">
@@ -2333,12 +2326,12 @@
         <f>'07_GE2_School_Outreach'!$C$10</f>
         <v/>
       </c>
-      <c r="G19" s="67" t="inlineStr">
+      <c r="G19" s="68" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="H19" s="68" t="inlineStr">
+      <c r="H19" s="69" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
@@ -2378,12 +2371,12 @@
         <f>'07_GE2_School_Outreach'!$C$12</f>
         <v/>
       </c>
-      <c r="G20" s="70" t="inlineStr">
+      <c r="G20" s="71" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
       </c>
-      <c r="H20" s="71" t="inlineStr">
+      <c r="H20" s="72" t="inlineStr">
         <is>
           <t>Baseline</t>
         </is>
@@ -2484,10 +2477,10 @@
         <f>COUNT('05_Daily_Log'!$D$8:$D$21)</f>
         <v/>
       </c>
-      <c r="G24" s="67" t="n">
+      <c r="G24" s="68" t="n">
         <v>14</v>
       </c>
-      <c r="H24" s="68" t="n">
+      <c r="H24" s="69" t="n">
         <v>12</v>
       </c>
       <c r="I24" s="47" t="inlineStr">
@@ -2503,7 +2496,7 @@
     <row r="25">
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Links in 09_UTM_Register that build a tagged URL</t>
+          <t>Sprint codes created in the live UTM register</t>
         </is>
       </c>
       <c r="C25" s="37" t="inlineStr">
@@ -2522,13 +2515,13 @@
         </is>
       </c>
       <c r="F25" s="24">
-        <f>COUNTIF('09_UTM_Register'!$H$7:$H$19,"?*")</f>
-        <v/>
-      </c>
-      <c r="G25" s="67" t="n">
+        <f>COUNTIF('09_UTM_Register'!$H$13:$H$25,"Y")</f>
+        <v/>
+      </c>
+      <c r="G25" s="68" t="n">
         <v>13</v>
       </c>
-      <c r="H25" s="68" t="n">
+      <c r="H25" s="69" t="n">
         <v>13</v>
       </c>
       <c r="I25" s="47" t="inlineStr">
@@ -2562,17 +2555,17 @@
           <t>Gradesmatch tech</t>
         </is>
       </c>
-      <c r="F26" s="72" t="inlineStr">
+      <c r="F26" s="73" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G26" s="73" t="inlineStr">
+      <c r="G26" s="74" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H26" s="74" t="inlineStr">
+      <c r="H26" s="75" t="inlineStr">
         <is>
           <t>Any miss</t>
         </is>
@@ -2609,17 +2602,17 @@
           <t>Schools Coordinator</t>
         </is>
       </c>
-      <c r="F27" s="72" t="inlineStr">
+      <c r="F27" s="73" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G27" s="73" t="inlineStr">
+      <c r="G27" s="74" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H27" s="74" t="inlineStr">
+      <c r="H27" s="75" t="inlineStr">
         <is>
           <t>Any miss</t>
         </is>
@@ -2656,17 +2649,17 @@
           <t>Campaign Lead</t>
         </is>
       </c>
-      <c r="F28" s="72" t="inlineStr">
+      <c r="F28" s="73" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="G28" s="73" t="inlineStr">
+      <c r="G28" s="74" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="H28" s="74" t="inlineStr">
+      <c r="H28" s="75" t="inlineStr">
         <is>
           <t>Any miss</t>
         </is>
@@ -2780,7 +2773,7 @@
         <f>'05_Daily_Log'!$L$22</f>
         <v/>
       </c>
-      <c r="D7" s="67">
+      <c r="D7" s="68">
         <f>'03_Sprint_Drivers'!$C$14</f>
         <v/>
       </c>
@@ -2804,7 +2797,7 @@
         <f>IFERROR(('05_Daily_Log'!$D$22+'07_GE2_School_Outreach'!$C$23)/'05_Daily_Log'!$L$22,0)</f>
         <v/>
       </c>
-      <c r="D8" s="65">
+      <c r="D8" s="66">
         <f>'03_Sprint_Drivers'!$C$26</f>
         <v/>
       </c>
@@ -2828,7 +2821,7 @@
         <f>'06_GE1_Paid_Media'!$C$11</f>
         <v/>
       </c>
-      <c r="D9" s="65">
+      <c r="D9" s="66">
         <f>'03_Sprint_Drivers'!$C$26*2</f>
         <v/>
       </c>
@@ -2852,7 +2845,7 @@
         <f>'07_GE2_School_Outreach'!$C$24</f>
         <v/>
       </c>
-      <c r="D10" s="65">
+      <c r="D10" s="66">
         <f>'03_Sprint_Drivers'!$C$26*2</f>
         <v/>
       </c>
@@ -2876,7 +2869,7 @@
         <f>IF(OR(AND(ISNUMBER('06_GE1_Paid_Media'!$C$11),'06_GE1_Paid_Media'!$C$11&lt;='03_Sprint_Drivers'!$C$26,'06_GE1_Paid_Media'!$C$11&gt;0),AND(ISNUMBER('07_GE2_School_Outreach'!$C$24),'07_GE2_School_Outreach'!$C$24&lt;='03_Sprint_Drivers'!$C$26,'07_GE2_School_Outreach'!$C$24&gt;0)),1,0)</f>
         <v/>
       </c>
-      <c r="D11" s="67" t="n">
+      <c r="D11" s="68" t="n">
         <v>1</v>
       </c>
       <c r="E11" s="43">
@@ -2899,7 +2892,7 @@
         <f>'05_Daily_Log'!$D$22</f>
         <v/>
       </c>
-      <c r="D12" s="65">
+      <c r="D12" s="66">
         <f>'03_Sprint_Drivers'!$C$13</f>
         <v/>
       </c>
@@ -2923,7 +2916,7 @@
         <f>COUNT('05_Daily_Log'!$D$8:$D$21)</f>
         <v/>
       </c>
-      <c r="D13" s="67" t="n">
+      <c r="D13" s="68" t="n">
         <v>14</v>
       </c>
       <c r="E13" s="43">
@@ -2946,7 +2939,7 @@
         <f>COUNTIF(E7:E13,"PASS")</f>
         <v/>
       </c>
-      <c r="D15" s="73" t="n">
+      <c r="D15" s="74" t="n">
         <v>7</v>
       </c>
       <c r="F15" s="2" t="inlineStr">

</xml_diff>